<commit_message>
mame: prepare help sample data for step 3
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/08_mame_evolvepro_raw.xlsx
+++ b/src-tauri/samples/mame/08_mame_evolvepro_raw.xlsx
@@ -441,37 +441,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S65T</t>
+          <t>65A</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.85</v>
+        <v>3.11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Y66H</t>
+          <t>203Y</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.48</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T203Y</t>
+          <t>65T</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.33</v>
+        <v>1.85</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>F64L</t>
+          <t>64L</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -481,7 +481,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A206K</t>
+          <t>206K</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -491,11 +491,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S65A</t>
+          <t>66H</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3.11</v>
+        <v>0.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v0.16.43: a representative that could actually be picked
Stop the bundled sample electing an AMBIGUOUS well as a variant representative, and report sample files that resolve but are not on disk instead of failing later in step 4. See CHANGELOG for detail.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/08_mame_evolvepro_raw.xlsx
+++ b/src-tauri/samples/mame/08_mame_evolvepro_raw.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,40 +481,50 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>150A</t>
+          <t>239A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>163A</t>
+          <t>150A</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.88</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>97A</t>
+          <t>163A</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.6233333333333334</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>97A</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.6233333333333334</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>190A</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>0.47</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.16.44: every variant recovered on one of three reads
Apply the PASS-only representative rule to every variant: each defect lands on a single barcode so a passing copy always represents the variant, no representative comes from the fallback path, and all eight verdict classes remain in the replicate comparison. See CHANGELOG for detail.
</commit_message>
<xml_diff>
--- a/src-tauri/samples/mame/08_mame_evolvepro_raw.xlsx
+++ b/src-tauri/samples/mame/08_mame_evolvepro_raw.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,70 +461,130 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>124A</t>
+          <t>227V</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.54</v>
+        <v>1.68</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>175A</t>
+          <t>124A</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.33</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>239A</t>
+          <t>205A</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1.2</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>150A</t>
+          <t>175A</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.19</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>163A</t>
+          <t>239A</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.88</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>97A</t>
+          <t>150A</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.6233333333333334</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>200A</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>215A</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.9500000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>163A</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>210A</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>97A</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.6233333333333334</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>235A</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5499999999999999</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>190A</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B17" t="n">
         <v>0.47</v>
       </c>
     </row>

</xml_diff>